<commit_message>
Update master data mappings based on user's new Excel changes
</commit_message>
<xml_diff>
--- a/StudentMasterDatalocal system.xlsx
+++ b/StudentMasterDatalocal system.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="160">
   <si>
     <t>branch_id</t>
   </si>
@@ -296,9 +296,6 @@
     <t>enrolled academic year</t>
   </si>
   <si>
-    <t>from CSV</t>
-  </si>
-  <si>
     <t>grade</t>
   </si>
   <si>
@@ -489,6 +486,21 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>student_type</t>
+  </si>
+  <si>
+    <t>Sinhalese</t>
+  </si>
+  <si>
+    <t>Muslim</t>
+  </si>
+  <si>
+    <t>Tamil</t>
+  </si>
+  <si>
+    <t>Bergur</t>
   </si>
 </sst>
 </file>
@@ -2453,7 +2465,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AH100"/>
+  <dimension ref="A1:AI100"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.6640625" customWidth="1"/>
@@ -2468,27 +2480,27 @@
     <col min="10" max="10" width="19.109375" customWidth="1"/>
     <col min="11" max="11" width="18.77734375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" customWidth="1"/>
-    <col min="14" max="15" width="18.6640625" customWidth="1"/>
-    <col min="16" max="17" width="26" customWidth="1"/>
-    <col min="18" max="18" width="9.6640625" customWidth="1"/>
-    <col min="19" max="19" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="12.109375" customWidth="1"/>
-    <col min="24" max="24" width="16.5546875" customWidth="1"/>
-    <col min="25" max="25" width="18" customWidth="1"/>
-    <col min="26" max="26" width="7.6640625" customWidth="1"/>
-    <col min="27" max="27" width="9.109375" customWidth="1"/>
-    <col min="28" max="28" width="13.109375" customWidth="1"/>
-    <col min="29" max="29" width="10.5546875" customWidth="1"/>
-    <col min="30" max="30" width="9.33203125" customWidth="1"/>
-    <col min="31" max="31" width="7.88671875" customWidth="1"/>
-    <col min="32" max="33" width="19.88671875" customWidth="1"/>
-    <col min="34" max="34" width="14.33203125" customWidth="1"/>
+    <col min="13" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="16" width="18.6640625" customWidth="1"/>
+    <col min="17" max="18" width="26" customWidth="1"/>
+    <col min="19" max="19" width="9.6640625" customWidth="1"/>
+    <col min="20" max="20" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="12.109375" customWidth="1"/>
+    <col min="25" max="25" width="16.5546875" customWidth="1"/>
+    <col min="26" max="26" width="18" customWidth="1"/>
+    <col min="27" max="27" width="7.6640625" customWidth="1"/>
+    <col min="28" max="28" width="9.109375" customWidth="1"/>
+    <col min="29" max="29" width="13.109375" customWidth="1"/>
+    <col min="30" max="30" width="10.5546875" customWidth="1"/>
+    <col min="31" max="31" width="9.33203125" customWidth="1"/>
+    <col min="32" max="32" width="7.88671875" customWidth="1"/>
+    <col min="33" max="34" width="19.88671875" customWidth="1"/>
+    <col min="35" max="35" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="14.4">
+    <row r="1" spans="1:35" ht="14.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2529,70 +2541,73 @@
         <v>42</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="T1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="U1" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="X1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="14.4">
+    <row r="2" spans="1:35" ht="14.4">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2613,60 +2628,67 @@
       <c r="L2" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="3">
+        <v>1</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="3">
+      <c r="O2" s="3">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="R2" s="3">
+      <c r="Q2" s="3">
         <v>1</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="R2" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="S2" s="3">
+        <v>1</v>
+      </c>
+      <c r="T2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="3">
+      <c r="U2" s="3">
         <v>1</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="3">
+      <c r="W2" s="3">
         <v>1</v>
       </c>
-      <c r="W2" s="9" t="s">
+      <c r="X2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="X2" s="3"/>
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="9" t="s">
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="AE2" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="AF2" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="AD2" s="3"/>
-      <c r="AE2" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="AF2" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="AG2" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="AH2" s="3" t="s">
+      <c r="AH2" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="AI2" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="14.4">
+    <row r="3" spans="1:35" ht="14.4">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -2682,27 +2704,31 @@
       <c r="K3" s="6"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3">
         <v>2</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3">
+      <c r="Q3" s="3">
         <v>2</v>
       </c>
-      <c r="S3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="T3" s="3">
+      <c r="R3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="S3" s="3">
         <v>2</v>
       </c>
-      <c r="U3" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="V3" s="3"/>
+      <c r="T3" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="U3" s="3">
+        <v>2</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>102</v>
+      </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
@@ -2711,16 +2737,19 @@
       <c r="AB3" s="3"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
-      <c r="AE3" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="AF3" s="3"/>
-      <c r="AG3" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="AH3" s="3"/>
-    </row>
-    <row r="4" spans="1:34" ht="14.4">
+      <c r="AE3" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="AF3" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="AI3" s="3"/>
+    </row>
+    <row r="4" spans="1:35" ht="14.4">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2734,27 +2763,31 @@
       <c r="K4" s="6"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-      <c r="N4" s="3">
+      <c r="N4" s="3"/>
+      <c r="O4" s="3">
         <v>3</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3">
+      <c r="Q4" s="3">
         <v>3</v>
       </c>
-      <c r="S4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="T4" s="3">
+      <c r="R4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="3">
         <v>3</v>
       </c>
-      <c r="U4" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="V4" s="3"/>
+      <c r="T4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="U4" s="3">
+        <v>3</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>103</v>
+      </c>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
@@ -2763,16 +2796,19 @@
       <c r="AB4" s="3"/>
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
-      <c r="AE4" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="AF4" s="3"/>
-      <c r="AG4" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="AH4" s="3"/>
-    </row>
-    <row r="5" spans="1:34" ht="14.4">
+      <c r="AE4" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="AF4" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="AI4" s="3"/>
+    </row>
+    <row r="5" spans="1:35" ht="14.4">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -2790,19 +2826,19 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
-      <c r="R5" s="3">
+      <c r="R5" s="3"/>
+      <c r="S5" s="3">
         <v>4</v>
       </c>
-      <c r="S5" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="T5" s="3">
+      <c r="T5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="U5" s="3">
         <v>4</v>
       </c>
-      <c r="U5" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="V5" s="3"/>
+      <c r="V5" s="3" t="s">
+        <v>104</v>
+      </c>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
       <c r="Y5" s="3"/>
@@ -2811,12 +2847,15 @@
       <c r="AB5" s="3"/>
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
-      <c r="AE5" s="3"/>
+      <c r="AE5" s="3" t="s">
+        <v>159</v>
+      </c>
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
-    </row>
-    <row r="6" spans="1:34" ht="14.4">
+      <c r="AI5" s="3"/>
+    </row>
+    <row r="6" spans="1:35" ht="14.4">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -2834,19 +2873,19 @@
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-      <c r="R6" s="3">
+      <c r="R6" s="3"/>
+      <c r="S6" s="3">
         <v>5</v>
       </c>
-      <c r="S6" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="T6" s="3">
+      <c r="T6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="U6" s="3">
         <v>5</v>
       </c>
-      <c r="U6" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="V6" s="3"/>
+      <c r="V6" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
@@ -2859,8 +2898,9 @@
       <c r="AF6" s="3"/>
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
-    </row>
-    <row r="7" spans="1:34" ht="14.4">
+      <c r="AI6" s="3"/>
+    </row>
+    <row r="7" spans="1:35" ht="14.4">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -2878,19 +2918,19 @@
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
-      <c r="R7" s="3">
+      <c r="R7" s="3"/>
+      <c r="S7" s="3">
         <v>6</v>
       </c>
-      <c r="S7" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="T7" s="3">
+      <c r="T7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="U7" s="3">
         <v>6</v>
       </c>
-      <c r="U7" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="V7" s="3"/>
+      <c r="V7" s="3" t="s">
+        <v>106</v>
+      </c>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
       <c r="Y7" s="3"/>
@@ -2903,8 +2943,9 @@
       <c r="AF7" s="3"/>
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
-    </row>
-    <row r="8" spans="1:34" ht="14.4">
+      <c r="AI7" s="3"/>
+    </row>
+    <row r="8" spans="1:35" ht="14.4">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -2922,19 +2963,19 @@
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
-      <c r="R8" s="3">
+      <c r="R8" s="3"/>
+      <c r="S8" s="3">
         <v>7</v>
       </c>
-      <c r="S8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="T8" s="3">
+      <c r="T8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="U8" s="3">
         <v>7</v>
       </c>
-      <c r="U8" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="V8" s="3"/>
+      <c r="V8" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
       <c r="Y8" s="3"/>
@@ -2947,8 +2988,9 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
-    </row>
-    <row r="9" spans="1:34" ht="14.4">
+      <c r="AI8" s="3"/>
+    </row>
+    <row r="9" spans="1:35" ht="14.4">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -2966,19 +3008,19 @@
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
-      <c r="R9" s="3">
+      <c r="R9" s="3"/>
+      <c r="S9" s="3">
         <v>8</v>
       </c>
-      <c r="S9" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="T9" s="3">
+      <c r="T9" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="U9" s="3">
         <v>8</v>
       </c>
-      <c r="U9" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="V9" s="3"/>
+      <c r="V9" s="3" t="s">
+        <v>108</v>
+      </c>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
@@ -2991,8 +3033,9 @@
       <c r="AF9" s="3"/>
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
-    </row>
-    <row r="10" spans="1:34" ht="14.4">
+      <c r="AI9" s="3"/>
+    </row>
+    <row r="10" spans="1:35" ht="14.4">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -3010,19 +3053,19 @@
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
-      <c r="R10" s="3">
+      <c r="R10" s="3"/>
+      <c r="S10" s="3">
         <v>9</v>
       </c>
-      <c r="S10" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T10" s="3">
+      <c r="T10" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="U10" s="3">
         <v>9</v>
       </c>
-      <c r="U10" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="V10" s="3"/>
+      <c r="V10" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
@@ -3035,8 +3078,9 @@
       <c r="AF10" s="3"/>
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
-    </row>
-    <row r="11" spans="1:34" ht="14.4">
+      <c r="AI10" s="3"/>
+    </row>
+    <row r="11" spans="1:35" ht="14.4">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -3054,19 +3098,19 @@
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
-      <c r="R11" s="3">
+      <c r="R11" s="3"/>
+      <c r="S11" s="3">
         <v>10</v>
       </c>
-      <c r="S11" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="T11" s="3">
+      <c r="T11" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="U11" s="3">
         <v>10</v>
       </c>
-      <c r="U11" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="V11" s="3"/>
+      <c r="V11" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
@@ -3079,8 +3123,9 @@
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
-    </row>
-    <row r="12" spans="1:34" ht="14.4">
+      <c r="AI11" s="3"/>
+    </row>
+    <row r="12" spans="1:35" ht="14.4">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -3100,13 +3145,13 @@
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
-      <c r="T12" s="3">
+      <c r="T12" s="3"/>
+      <c r="U12" s="3">
         <v>11</v>
       </c>
-      <c r="U12" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="V12" s="3"/>
+      <c r="V12" s="3" t="s">
+        <v>111</v>
+      </c>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
       <c r="Y12" s="3"/>
@@ -3119,8 +3164,9 @@
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
-    </row>
-    <row r="13" spans="1:34" ht="14.4">
+      <c r="AI12" s="3"/>
+    </row>
+    <row r="13" spans="1:35" ht="14.4">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3140,13 +3186,13 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
-      <c r="T13" s="3">
+      <c r="T13" s="3"/>
+      <c r="U13" s="3">
         <v>12</v>
       </c>
-      <c r="U13" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="V13" s="3"/>
+      <c r="V13" s="3" t="s">
+        <v>112</v>
+      </c>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="3"/>
@@ -3159,8 +3205,9 @@
       <c r="AF13" s="3"/>
       <c r="AG13" s="3"/>
       <c r="AH13" s="3"/>
-    </row>
-    <row r="14" spans="1:34" ht="14.4">
+      <c r="AI13" s="3"/>
+    </row>
+    <row r="14" spans="1:35" ht="14.4">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -3180,13 +3227,13 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
-      <c r="T14" s="3">
+      <c r="T14" s="3"/>
+      <c r="U14" s="3">
         <v>13</v>
       </c>
-      <c r="U14" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="V14" s="3"/>
+      <c r="V14" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
@@ -3199,8 +3246,9 @@
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
-    </row>
-    <row r="15" spans="1:34" ht="14.4">
+      <c r="AI14" s="3"/>
+    </row>
+    <row r="15" spans="1:35" ht="14.4">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -3220,13 +3268,13 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
-      <c r="T15" s="3">
+      <c r="T15" s="3"/>
+      <c r="U15" s="3">
         <v>14</v>
       </c>
-      <c r="U15" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="V15" s="3"/>
+      <c r="V15" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
       <c r="Y15" s="3"/>
@@ -3239,8 +3287,9 @@
       <c r="AF15" s="3"/>
       <c r="AG15" s="3"/>
       <c r="AH15" s="3"/>
-    </row>
-    <row r="16" spans="1:34" ht="14.4">
+      <c r="AI15" s="3"/>
+    </row>
+    <row r="16" spans="1:35" ht="14.4">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -3260,13 +3309,13 @@
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
-      <c r="T16" s="3">
+      <c r="T16" s="3"/>
+      <c r="U16" s="3">
         <v>15</v>
       </c>
-      <c r="U16" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="V16" s="3"/>
+      <c r="V16" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
       <c r="Y16" s="3"/>
@@ -3279,8 +3328,9 @@
       <c r="AF16" s="3"/>
       <c r="AG16" s="3"/>
       <c r="AH16" s="3"/>
-    </row>
-    <row r="17" spans="1:34" ht="14.4">
+      <c r="AI16" s="3"/>
+    </row>
+    <row r="17" spans="1:35" ht="14.4">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3300,13 +3350,13 @@
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
-      <c r="T17" s="3">
+      <c r="T17" s="3"/>
+      <c r="U17" s="3">
         <v>16</v>
       </c>
-      <c r="U17" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="V17" s="3"/>
+      <c r="V17" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
       <c r="Y17" s="3"/>
@@ -3319,8 +3369,9 @@
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
       <c r="AH17" s="3"/>
-    </row>
-    <row r="18" spans="1:34" ht="14.4">
+      <c r="AI17" s="3"/>
+    </row>
+    <row r="18" spans="1:35" ht="14.4">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -3340,13 +3391,13 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
-      <c r="T18" s="3">
+      <c r="T18" s="3"/>
+      <c r="U18" s="3">
         <v>17</v>
       </c>
-      <c r="U18" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="V18" s="3"/>
+      <c r="V18" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
@@ -3359,8 +3410,9 @@
       <c r="AF18" s="3"/>
       <c r="AG18" s="3"/>
       <c r="AH18" s="3"/>
-    </row>
-    <row r="19" spans="1:34" ht="14.4">
+      <c r="AI18" s="3"/>
+    </row>
+    <row r="19" spans="1:35" ht="14.4">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -3380,13 +3432,13 @@
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
-      <c r="T19" s="3">
+      <c r="T19" s="3"/>
+      <c r="U19" s="3">
         <v>18</v>
       </c>
-      <c r="U19" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="V19" s="3"/>
+      <c r="V19" s="3" t="s">
+        <v>118</v>
+      </c>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
@@ -3399,8 +3451,9 @@
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
-    </row>
-    <row r="20" spans="1:34" ht="14.4">
+      <c r="AI19" s="3"/>
+    </row>
+    <row r="20" spans="1:35" ht="14.4">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -3420,13 +3473,13 @@
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
       <c r="S20" s="3"/>
-      <c r="T20" s="3">
+      <c r="T20" s="3"/>
+      <c r="U20" s="3">
         <v>19</v>
       </c>
-      <c r="U20" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="V20" s="3"/>
+      <c r="V20" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
@@ -3439,8 +3492,9 @@
       <c r="AF20" s="3"/>
       <c r="AG20" s="3"/>
       <c r="AH20" s="3"/>
-    </row>
-    <row r="21" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI20" s="3"/>
+    </row>
+    <row r="21" spans="1:35" ht="15.75" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -3460,13 +3514,13 @@
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
       <c r="S21" s="3"/>
-      <c r="T21" s="3">
+      <c r="T21" s="3"/>
+      <c r="U21" s="3">
         <v>20</v>
       </c>
-      <c r="U21" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="V21" s="3"/>
+      <c r="V21" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
       <c r="Y21" s="3"/>
@@ -3479,8 +3533,9 @@
       <c r="AF21" s="3"/>
       <c r="AG21" s="3"/>
       <c r="AH21" s="3"/>
-    </row>
-    <row r="22" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI21" s="3"/>
+    </row>
+    <row r="22" spans="1:35" ht="15.75" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -3500,13 +3555,13 @@
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
       <c r="S22" s="3"/>
-      <c r="T22" s="3">
+      <c r="T22" s="3"/>
+      <c r="U22" s="3">
         <v>21</v>
       </c>
-      <c r="U22" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="V22" s="3"/>
+      <c r="V22" s="3" t="s">
+        <v>121</v>
+      </c>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
       <c r="Y22" s="3"/>
@@ -3519,8 +3574,9 @@
       <c r="AF22" s="3"/>
       <c r="AG22" s="3"/>
       <c r="AH22" s="3"/>
-    </row>
-    <row r="23" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI22" s="3"/>
+    </row>
+    <row r="23" spans="1:35" ht="15.75" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -3540,13 +3596,13 @@
       <c r="Q23" s="3"/>
       <c r="R23" s="3"/>
       <c r="S23" s="3"/>
-      <c r="T23" s="3">
+      <c r="T23" s="3"/>
+      <c r="U23" s="3">
         <v>22</v>
       </c>
-      <c r="U23" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="V23" s="3"/>
+      <c r="V23" s="3" t="s">
+        <v>122</v>
+      </c>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
       <c r="Y23" s="3"/>
@@ -3559,8 +3615,9 @@
       <c r="AF23" s="3"/>
       <c r="AG23" s="3"/>
       <c r="AH23" s="3"/>
-    </row>
-    <row r="24" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI23" s="3"/>
+    </row>
+    <row r="24" spans="1:35" ht="15.75" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -3580,13 +3637,13 @@
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
       <c r="S24" s="3"/>
-      <c r="T24" s="3">
+      <c r="T24" s="3"/>
+      <c r="U24" s="3">
         <v>23</v>
       </c>
-      <c r="U24" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="V24" s="3"/>
+      <c r="V24" s="3" t="s">
+        <v>123</v>
+      </c>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
       <c r="Y24" s="3"/>
@@ -3599,8 +3656,9 @@
       <c r="AF24" s="3"/>
       <c r="AG24" s="3"/>
       <c r="AH24" s="3"/>
-    </row>
-    <row r="25" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI24" s="3"/>
+    </row>
+    <row r="25" spans="1:35" ht="15.75" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -3620,13 +3678,13 @@
       <c r="Q25" s="3"/>
       <c r="R25" s="3"/>
       <c r="S25" s="3"/>
-      <c r="T25" s="3">
+      <c r="T25" s="3"/>
+      <c r="U25" s="3">
         <v>24</v>
       </c>
-      <c r="U25" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="V25" s="3"/>
+      <c r="V25" s="3" t="s">
+        <v>124</v>
+      </c>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
       <c r="Y25" s="3"/>
@@ -3639,8 +3697,9 @@
       <c r="AF25" s="3"/>
       <c r="AG25" s="3"/>
       <c r="AH25" s="3"/>
-    </row>
-    <row r="26" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI25" s="3"/>
+    </row>
+    <row r="26" spans="1:35" ht="15.75" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -3660,13 +3719,13 @@
       <c r="Q26" s="3"/>
       <c r="R26" s="3"/>
       <c r="S26" s="3"/>
-      <c r="T26" s="3">
+      <c r="T26" s="3"/>
+      <c r="U26" s="3">
         <v>25</v>
       </c>
-      <c r="U26" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="V26" s="3"/>
+      <c r="V26" s="3" t="s">
+        <v>125</v>
+      </c>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
       <c r="Y26" s="3"/>
@@ -3679,8 +3738,9 @@
       <c r="AF26" s="3"/>
       <c r="AG26" s="3"/>
       <c r="AH26" s="3"/>
-    </row>
-    <row r="27" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI26" s="3"/>
+    </row>
+    <row r="27" spans="1:35" ht="15.75" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -3700,13 +3760,13 @@
       <c r="Q27" s="3"/>
       <c r="R27" s="3"/>
       <c r="S27" s="3"/>
-      <c r="T27" s="3">
+      <c r="T27" s="3"/>
+      <c r="U27" s="3">
         <v>26</v>
       </c>
-      <c r="U27" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="V27" s="3"/>
+      <c r="V27" s="3" t="s">
+        <v>126</v>
+      </c>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
       <c r="Y27" s="3"/>
@@ -3719,8 +3779,9 @@
       <c r="AF27" s="3"/>
       <c r="AG27" s="3"/>
       <c r="AH27" s="3"/>
-    </row>
-    <row r="28" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI27" s="3"/>
+    </row>
+    <row r="28" spans="1:35" ht="15.75" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -3740,13 +3801,13 @@
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
       <c r="S28" s="3"/>
-      <c r="T28" s="3">
+      <c r="T28" s="3"/>
+      <c r="U28" s="3">
         <v>27</v>
       </c>
-      <c r="U28" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="V28" s="3"/>
+      <c r="V28" s="3" t="s">
+        <v>127</v>
+      </c>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
       <c r="Y28" s="3"/>
@@ -3759,8 +3820,9 @@
       <c r="AF28" s="3"/>
       <c r="AG28" s="3"/>
       <c r="AH28" s="3"/>
-    </row>
-    <row r="29" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI28" s="3"/>
+    </row>
+    <row r="29" spans="1:35" ht="15.75" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -3780,13 +3842,13 @@
       <c r="Q29" s="3"/>
       <c r="R29" s="3"/>
       <c r="S29" s="3"/>
-      <c r="T29" s="3">
+      <c r="T29" s="3"/>
+      <c r="U29" s="3">
         <v>28</v>
       </c>
-      <c r="U29" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="V29" s="3"/>
+      <c r="V29" s="3" t="s">
+        <v>128</v>
+      </c>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
@@ -3799,8 +3861,9 @@
       <c r="AF29" s="3"/>
       <c r="AG29" s="3"/>
       <c r="AH29" s="3"/>
-    </row>
-    <row r="30" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI29" s="3"/>
+    </row>
+    <row r="30" spans="1:35" ht="15.75" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -3820,13 +3883,13 @@
       <c r="Q30" s="3"/>
       <c r="R30" s="3"/>
       <c r="S30" s="3"/>
-      <c r="T30" s="3">
+      <c r="T30" s="3"/>
+      <c r="U30" s="3">
         <v>29</v>
       </c>
-      <c r="U30" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="V30" s="3"/>
+      <c r="V30" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
       <c r="Y30" s="3"/>
@@ -3839,8 +3902,9 @@
       <c r="AF30" s="3"/>
       <c r="AG30" s="3"/>
       <c r="AH30" s="3"/>
-    </row>
-    <row r="31" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI30" s="3"/>
+    </row>
+    <row r="31" spans="1:35" ht="15.75" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -3860,13 +3924,13 @@
       <c r="Q31" s="3"/>
       <c r="R31" s="3"/>
       <c r="S31" s="3"/>
-      <c r="T31" s="3">
+      <c r="T31" s="3"/>
+      <c r="U31" s="3">
         <v>30</v>
       </c>
-      <c r="U31" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="V31" s="3"/>
+      <c r="V31" s="3" t="s">
+        <v>130</v>
+      </c>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
       <c r="Y31" s="3"/>
@@ -3879,8 +3943,9 @@
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
       <c r="AH31" s="3"/>
-    </row>
-    <row r="32" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI31" s="3"/>
+    </row>
+    <row r="32" spans="1:35" ht="15.75" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -3900,13 +3965,13 @@
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
       <c r="S32" s="3"/>
-      <c r="T32" s="3">
+      <c r="T32" s="3"/>
+      <c r="U32" s="3">
         <v>31</v>
       </c>
-      <c r="U32" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="V32" s="3"/>
+      <c r="V32" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
       <c r="Y32" s="3"/>
@@ -3919,8 +3984,9 @@
       <c r="AF32" s="3"/>
       <c r="AG32" s="3"/>
       <c r="AH32" s="3"/>
-    </row>
-    <row r="33" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI32" s="3"/>
+    </row>
+    <row r="33" spans="1:35" ht="15.75" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -3940,13 +4006,13 @@
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
-      <c r="T33" s="3">
+      <c r="T33" s="3"/>
+      <c r="U33" s="3">
         <v>32</v>
       </c>
-      <c r="U33" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="V33" s="3"/>
+      <c r="V33" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
       <c r="Y33" s="3"/>
@@ -3959,8 +4025,9 @@
       <c r="AF33" s="3"/>
       <c r="AG33" s="3"/>
       <c r="AH33" s="3"/>
-    </row>
-    <row r="34" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI33" s="3"/>
+    </row>
+    <row r="34" spans="1:35" ht="15.75" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -3980,13 +4047,13 @@
       <c r="Q34" s="3"/>
       <c r="R34" s="3"/>
       <c r="S34" s="3"/>
-      <c r="T34" s="3">
+      <c r="T34" s="3"/>
+      <c r="U34" s="3">
         <v>33</v>
       </c>
-      <c r="U34" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="V34" s="3"/>
+      <c r="V34" s="3" t="s">
+        <v>133</v>
+      </c>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
@@ -3999,8 +4066,9 @@
       <c r="AF34" s="3"/>
       <c r="AG34" s="3"/>
       <c r="AH34" s="3"/>
-    </row>
-    <row r="35" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI34" s="3"/>
+    </row>
+    <row r="35" spans="1:35" ht="15.75" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -4020,13 +4088,13 @@
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
       <c r="S35" s="3"/>
-      <c r="T35" s="3">
+      <c r="T35" s="3"/>
+      <c r="U35" s="3">
         <v>34</v>
       </c>
-      <c r="U35" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="V35" s="3"/>
+      <c r="V35" s="3" t="s">
+        <v>134</v>
+      </c>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
       <c r="Y35" s="3"/>
@@ -4039,8 +4107,9 @@
       <c r="AF35" s="3"/>
       <c r="AG35" s="3"/>
       <c r="AH35" s="3"/>
-    </row>
-    <row r="36" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI35" s="3"/>
+    </row>
+    <row r="36" spans="1:35" ht="15.75" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -4060,13 +4129,13 @@
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
       <c r="S36" s="3"/>
-      <c r="T36" s="3">
+      <c r="T36" s="3"/>
+      <c r="U36" s="3">
         <v>35</v>
       </c>
-      <c r="U36" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="V36" s="3"/>
+      <c r="V36" s="3" t="s">
+        <v>135</v>
+      </c>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
@@ -4079,8 +4148,9 @@
       <c r="AF36" s="3"/>
       <c r="AG36" s="3"/>
       <c r="AH36" s="3"/>
-    </row>
-    <row r="37" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI36" s="3"/>
+    </row>
+    <row r="37" spans="1:35" ht="15.75" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -4100,13 +4170,13 @@
       <c r="Q37" s="3"/>
       <c r="R37" s="3"/>
       <c r="S37" s="3"/>
-      <c r="T37" s="3">
+      <c r="T37" s="3"/>
+      <c r="U37" s="3">
         <v>36</v>
       </c>
-      <c r="U37" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="V37" s="3"/>
+      <c r="V37" s="3" t="s">
+        <v>136</v>
+      </c>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
       <c r="Y37" s="3"/>
@@ -4119,8 +4189,9 @@
       <c r="AF37" s="3"/>
       <c r="AG37" s="3"/>
       <c r="AH37" s="3"/>
-    </row>
-    <row r="38" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI37" s="3"/>
+    </row>
+    <row r="38" spans="1:35" ht="15.75" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -4140,13 +4211,13 @@
       <c r="Q38" s="3"/>
       <c r="R38" s="3"/>
       <c r="S38" s="3"/>
-      <c r="T38" s="3">
+      <c r="T38" s="3"/>
+      <c r="U38" s="3">
         <v>37</v>
       </c>
-      <c r="U38" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="V38" s="3"/>
+      <c r="V38" s="3" t="s">
+        <v>137</v>
+      </c>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
@@ -4159,8 +4230,9 @@
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
-    </row>
-    <row r="39" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI38" s="3"/>
+    </row>
+    <row r="39" spans="1:35" ht="15.75" customHeight="1">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -4180,13 +4252,13 @@
       <c r="Q39" s="3"/>
       <c r="R39" s="3"/>
       <c r="S39" s="3"/>
-      <c r="T39" s="3">
+      <c r="T39" s="3"/>
+      <c r="U39" s="3">
         <v>38</v>
       </c>
-      <c r="U39" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="V39" s="3"/>
+      <c r="V39" s="3" t="s">
+        <v>138</v>
+      </c>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
       <c r="Y39" s="3"/>
@@ -4199,8 +4271,9 @@
       <c r="AF39" s="3"/>
       <c r="AG39" s="3"/>
       <c r="AH39" s="3"/>
-    </row>
-    <row r="40" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI39" s="3"/>
+    </row>
+    <row r="40" spans="1:35" ht="15.75" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -4220,13 +4293,13 @@
       <c r="Q40" s="3"/>
       <c r="R40" s="3"/>
       <c r="S40" s="3"/>
-      <c r="T40" s="3">
+      <c r="T40" s="3"/>
+      <c r="U40" s="3">
         <v>39</v>
       </c>
-      <c r="U40" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="V40" s="3"/>
+      <c r="V40" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
       <c r="Y40" s="3"/>
@@ -4239,8 +4312,9 @@
       <c r="AF40" s="3"/>
       <c r="AG40" s="3"/>
       <c r="AH40" s="3"/>
-    </row>
-    <row r="41" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI40" s="3"/>
+    </row>
+    <row r="41" spans="1:35" ht="15.75" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -4260,13 +4334,13 @@
       <c r="Q41" s="3"/>
       <c r="R41" s="3"/>
       <c r="S41" s="3"/>
-      <c r="T41" s="3">
+      <c r="T41" s="3"/>
+      <c r="U41" s="3">
         <v>40</v>
       </c>
-      <c r="U41" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="V41" s="3"/>
+      <c r="V41" s="3" t="s">
+        <v>140</v>
+      </c>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
@@ -4279,8 +4353,9 @@
       <c r="AF41" s="3"/>
       <c r="AG41" s="3"/>
       <c r="AH41" s="3"/>
-    </row>
-    <row r="42" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI41" s="3"/>
+    </row>
+    <row r="42" spans="1:35" ht="15.75" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -4300,13 +4375,13 @@
       <c r="Q42" s="3"/>
       <c r="R42" s="3"/>
       <c r="S42" s="3"/>
-      <c r="T42" s="3">
+      <c r="T42" s="3"/>
+      <c r="U42" s="3">
         <v>41</v>
       </c>
-      <c r="U42" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="V42" s="3"/>
+      <c r="V42" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
@@ -4319,8 +4394,9 @@
       <c r="AF42" s="3"/>
       <c r="AG42" s="3"/>
       <c r="AH42" s="3"/>
-    </row>
-    <row r="43" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI42" s="3"/>
+    </row>
+    <row r="43" spans="1:35" ht="15.75" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -4340,13 +4416,13 @@
       <c r="Q43" s="3"/>
       <c r="R43" s="3"/>
       <c r="S43" s="3"/>
-      <c r="T43" s="3">
+      <c r="T43" s="3"/>
+      <c r="U43" s="3">
         <v>42</v>
       </c>
-      <c r="U43" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="V43" s="3"/>
+      <c r="V43" s="3" t="s">
+        <v>142</v>
+      </c>
       <c r="W43" s="3"/>
       <c r="X43" s="3"/>
       <c r="Y43" s="3"/>
@@ -4359,8 +4435,9 @@
       <c r="AF43" s="3"/>
       <c r="AG43" s="3"/>
       <c r="AH43" s="3"/>
-    </row>
-    <row r="44" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI43" s="3"/>
+    </row>
+    <row r="44" spans="1:35" ht="15.75" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -4380,13 +4457,13 @@
       <c r="Q44" s="3"/>
       <c r="R44" s="3"/>
       <c r="S44" s="3"/>
-      <c r="T44" s="3">
+      <c r="T44" s="3"/>
+      <c r="U44" s="3">
         <v>43</v>
       </c>
-      <c r="U44" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="V44" s="3"/>
+      <c r="V44" s="3" t="s">
+        <v>143</v>
+      </c>
       <c r="W44" s="3"/>
       <c r="X44" s="3"/>
       <c r="Y44" s="3"/>
@@ -4399,8 +4476,9 @@
       <c r="AF44" s="3"/>
       <c r="AG44" s="3"/>
       <c r="AH44" s="3"/>
-    </row>
-    <row r="45" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI44" s="3"/>
+    </row>
+    <row r="45" spans="1:35" ht="15.75" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -4420,13 +4498,13 @@
       <c r="Q45" s="3"/>
       <c r="R45" s="3"/>
       <c r="S45" s="3"/>
-      <c r="T45" s="3">
+      <c r="T45" s="3"/>
+      <c r="U45" s="3">
         <v>44</v>
       </c>
-      <c r="U45" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="V45" s="3"/>
+      <c r="V45" s="3" t="s">
+        <v>144</v>
+      </c>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
       <c r="Y45" s="3"/>
@@ -4439,8 +4517,9 @@
       <c r="AF45" s="3"/>
       <c r="AG45" s="3"/>
       <c r="AH45" s="3"/>
-    </row>
-    <row r="46" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI45" s="3"/>
+    </row>
+    <row r="46" spans="1:35" ht="15.75" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -4460,13 +4539,13 @@
       <c r="Q46" s="3"/>
       <c r="R46" s="3"/>
       <c r="S46" s="3"/>
-      <c r="T46" s="3">
+      <c r="T46" s="3"/>
+      <c r="U46" s="3">
         <v>45</v>
       </c>
-      <c r="U46" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="V46" s="3"/>
+      <c r="V46" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
       <c r="Y46" s="3"/>
@@ -4479,8 +4558,9 @@
       <c r="AF46" s="3"/>
       <c r="AG46" s="3"/>
       <c r="AH46" s="3"/>
-    </row>
-    <row r="47" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI46" s="3"/>
+    </row>
+    <row r="47" spans="1:35" ht="15.75" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -4500,13 +4580,13 @@
       <c r="Q47" s="3"/>
       <c r="R47" s="3"/>
       <c r="S47" s="3"/>
-      <c r="T47" s="3">
+      <c r="T47" s="3"/>
+      <c r="U47" s="3">
         <v>46</v>
       </c>
-      <c r="U47" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="V47" s="3"/>
+      <c r="V47" s="3" t="s">
+        <v>146</v>
+      </c>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
       <c r="Y47" s="3"/>
@@ -4519,8 +4599,9 @@
       <c r="AF47" s="3"/>
       <c r="AG47" s="3"/>
       <c r="AH47" s="3"/>
-    </row>
-    <row r="48" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI47" s="3"/>
+    </row>
+    <row r="48" spans="1:35" ht="15.75" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -4540,13 +4621,13 @@
       <c r="Q48" s="3"/>
       <c r="R48" s="3"/>
       <c r="S48" s="3"/>
-      <c r="T48" s="3">
+      <c r="T48" s="3"/>
+      <c r="U48" s="3">
         <v>47</v>
       </c>
-      <c r="U48" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="V48" s="3"/>
+      <c r="V48" s="3" t="s">
+        <v>147</v>
+      </c>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
       <c r="Y48" s="3"/>
@@ -4559,8 +4640,9 @@
       <c r="AF48" s="3"/>
       <c r="AG48" s="3"/>
       <c r="AH48" s="3"/>
-    </row>
-    <row r="49" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI48" s="3"/>
+    </row>
+    <row r="49" spans="1:35" ht="15.75" customHeight="1">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -4595,8 +4677,9 @@
       <c r="AF49" s="3"/>
       <c r="AG49" s="3"/>
       <c r="AH49" s="3"/>
-    </row>
-    <row r="50" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI49" s="3"/>
+    </row>
+    <row r="50" spans="1:35" ht="15.75" customHeight="1">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -4631,8 +4714,9 @@
       <c r="AF50" s="3"/>
       <c r="AG50" s="3"/>
       <c r="AH50" s="3"/>
-    </row>
-    <row r="51" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI50" s="3"/>
+    </row>
+    <row r="51" spans="1:35" ht="15.75" customHeight="1">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -4667,8 +4751,9 @@
       <c r="AF51" s="3"/>
       <c r="AG51" s="3"/>
       <c r="AH51" s="3"/>
-    </row>
-    <row r="52" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI51" s="3"/>
+    </row>
+    <row r="52" spans="1:35" ht="15.75" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -4703,8 +4788,9 @@
       <c r="AF52" s="3"/>
       <c r="AG52" s="3"/>
       <c r="AH52" s="3"/>
-    </row>
-    <row r="53" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI52" s="3"/>
+    </row>
+    <row r="53" spans="1:35" ht="15.75" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -4739,8 +4825,9 @@
       <c r="AF53" s="3"/>
       <c r="AG53" s="3"/>
       <c r="AH53" s="3"/>
-    </row>
-    <row r="54" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI53" s="3"/>
+    </row>
+    <row r="54" spans="1:35" ht="15.75" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -4775,8 +4862,9 @@
       <c r="AF54" s="3"/>
       <c r="AG54" s="3"/>
       <c r="AH54" s="3"/>
-    </row>
-    <row r="55" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI54" s="3"/>
+    </row>
+    <row r="55" spans="1:35" ht="15.75" customHeight="1">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -4811,8 +4899,9 @@
       <c r="AF55" s="3"/>
       <c r="AG55" s="3"/>
       <c r="AH55" s="3"/>
-    </row>
-    <row r="56" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI55" s="3"/>
+    </row>
+    <row r="56" spans="1:35" ht="15.75" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -4847,8 +4936,9 @@
       <c r="AF56" s="3"/>
       <c r="AG56" s="3"/>
       <c r="AH56" s="3"/>
-    </row>
-    <row r="57" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI56" s="3"/>
+    </row>
+    <row r="57" spans="1:35" ht="15.75" customHeight="1">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -4883,8 +4973,9 @@
       <c r="AF57" s="3"/>
       <c r="AG57" s="3"/>
       <c r="AH57" s="3"/>
-    </row>
-    <row r="58" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI57" s="3"/>
+    </row>
+    <row r="58" spans="1:35" ht="15.75" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -4919,8 +5010,9 @@
       <c r="AF58" s="3"/>
       <c r="AG58" s="3"/>
       <c r="AH58" s="3"/>
-    </row>
-    <row r="59" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI58" s="3"/>
+    </row>
+    <row r="59" spans="1:35" ht="15.75" customHeight="1">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -4955,8 +5047,9 @@
       <c r="AF59" s="3"/>
       <c r="AG59" s="3"/>
       <c r="AH59" s="3"/>
-    </row>
-    <row r="60" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI59" s="3"/>
+    </row>
+    <row r="60" spans="1:35" ht="15.75" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -4991,8 +5084,9 @@
       <c r="AF60" s="3"/>
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
-    </row>
-    <row r="61" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI60" s="3"/>
+    </row>
+    <row r="61" spans="1:35" ht="15.75" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -5027,8 +5121,9 @@
       <c r="AF61" s="3"/>
       <c r="AG61" s="3"/>
       <c r="AH61" s="3"/>
-    </row>
-    <row r="62" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI61" s="3"/>
+    </row>
+    <row r="62" spans="1:35" ht="15.75" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -5063,8 +5158,9 @@
       <c r="AF62" s="3"/>
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
-    </row>
-    <row r="63" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI62" s="3"/>
+    </row>
+    <row r="63" spans="1:35" ht="15.75" customHeight="1">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -5099,8 +5195,9 @@
       <c r="AF63" s="3"/>
       <c r="AG63" s="3"/>
       <c r="AH63" s="3"/>
-    </row>
-    <row r="64" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI63" s="3"/>
+    </row>
+    <row r="64" spans="1:35" ht="15.75" customHeight="1">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -5135,8 +5232,9 @@
       <c r="AF64" s="3"/>
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
-    </row>
-    <row r="65" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI64" s="3"/>
+    </row>
+    <row r="65" spans="1:35" ht="15.75" customHeight="1">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -5171,8 +5269,9 @@
       <c r="AF65" s="3"/>
       <c r="AG65" s="3"/>
       <c r="AH65" s="3"/>
-    </row>
-    <row r="66" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI65" s="3"/>
+    </row>
+    <row r="66" spans="1:35" ht="15.75" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -5207,8 +5306,9 @@
       <c r="AF66" s="3"/>
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
-    </row>
-    <row r="67" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI66" s="3"/>
+    </row>
+    <row r="67" spans="1:35" ht="15.75" customHeight="1">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -5243,8 +5343,9 @@
       <c r="AF67" s="3"/>
       <c r="AG67" s="3"/>
       <c r="AH67" s="3"/>
-    </row>
-    <row r="68" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI67" s="3"/>
+    </row>
+    <row r="68" spans="1:35" ht="15.75" customHeight="1">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -5279,8 +5380,9 @@
       <c r="AF68" s="3"/>
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
-    </row>
-    <row r="69" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI68" s="3"/>
+    </row>
+    <row r="69" spans="1:35" ht="15.75" customHeight="1">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -5315,8 +5417,9 @@
       <c r="AF69" s="3"/>
       <c r="AG69" s="3"/>
       <c r="AH69" s="3"/>
-    </row>
-    <row r="70" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI69" s="3"/>
+    </row>
+    <row r="70" spans="1:35" ht="15.75" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -5351,8 +5454,9 @@
       <c r="AF70" s="3"/>
       <c r="AG70" s="3"/>
       <c r="AH70" s="3"/>
-    </row>
-    <row r="71" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI70" s="3"/>
+    </row>
+    <row r="71" spans="1:35" ht="15.75" customHeight="1">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -5387,8 +5491,9 @@
       <c r="AF71" s="3"/>
       <c r="AG71" s="3"/>
       <c r="AH71" s="3"/>
-    </row>
-    <row r="72" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI71" s="3"/>
+    </row>
+    <row r="72" spans="1:35" ht="15.75" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -5423,8 +5528,9 @@
       <c r="AF72" s="3"/>
       <c r="AG72" s="3"/>
       <c r="AH72" s="3"/>
-    </row>
-    <row r="73" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI72" s="3"/>
+    </row>
+    <row r="73" spans="1:35" ht="15.75" customHeight="1">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -5459,8 +5565,9 @@
       <c r="AF73" s="3"/>
       <c r="AG73" s="3"/>
       <c r="AH73" s="3"/>
-    </row>
-    <row r="74" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI73" s="3"/>
+    </row>
+    <row r="74" spans="1:35" ht="15.75" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -5495,8 +5602,9 @@
       <c r="AF74" s="3"/>
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
-    </row>
-    <row r="75" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI74" s="3"/>
+    </row>
+    <row r="75" spans="1:35" ht="15.75" customHeight="1">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -5531,8 +5639,9 @@
       <c r="AF75" s="3"/>
       <c r="AG75" s="3"/>
       <c r="AH75" s="3"/>
-    </row>
-    <row r="76" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI75" s="3"/>
+    </row>
+    <row r="76" spans="1:35" ht="15.75" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -5567,8 +5676,9 @@
       <c r="AF76" s="3"/>
       <c r="AG76" s="3"/>
       <c r="AH76" s="3"/>
-    </row>
-    <row r="77" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI76" s="3"/>
+    </row>
+    <row r="77" spans="1:35" ht="15.75" customHeight="1">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -5603,8 +5713,9 @@
       <c r="AF77" s="3"/>
       <c r="AG77" s="3"/>
       <c r="AH77" s="3"/>
-    </row>
-    <row r="78" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI77" s="3"/>
+    </row>
+    <row r="78" spans="1:35" ht="15.75" customHeight="1">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -5639,8 +5750,9 @@
       <c r="AF78" s="3"/>
       <c r="AG78" s="3"/>
       <c r="AH78" s="3"/>
-    </row>
-    <row r="79" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI78" s="3"/>
+    </row>
+    <row r="79" spans="1:35" ht="15.75" customHeight="1">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -5675,8 +5787,9 @@
       <c r="AF79" s="3"/>
       <c r="AG79" s="3"/>
       <c r="AH79" s="3"/>
-    </row>
-    <row r="80" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI79" s="3"/>
+    </row>
+    <row r="80" spans="1:35" ht="15.75" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -5711,8 +5824,9 @@
       <c r="AF80" s="3"/>
       <c r="AG80" s="3"/>
       <c r="AH80" s="3"/>
-    </row>
-    <row r="81" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI80" s="3"/>
+    </row>
+    <row r="81" spans="1:35" ht="15.75" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -5747,8 +5861,9 @@
       <c r="AF81" s="3"/>
       <c r="AG81" s="3"/>
       <c r="AH81" s="3"/>
-    </row>
-    <row r="82" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI81" s="3"/>
+    </row>
+    <row r="82" spans="1:35" ht="15.75" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -5783,8 +5898,9 @@
       <c r="AF82" s="3"/>
       <c r="AG82" s="3"/>
       <c r="AH82" s="3"/>
-    </row>
-    <row r="83" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI82" s="3"/>
+    </row>
+    <row r="83" spans="1:35" ht="15.75" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -5819,8 +5935,9 @@
       <c r="AF83" s="3"/>
       <c r="AG83" s="3"/>
       <c r="AH83" s="3"/>
-    </row>
-    <row r="84" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI83" s="3"/>
+    </row>
+    <row r="84" spans="1:35" ht="15.75" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -5855,8 +5972,9 @@
       <c r="AF84" s="3"/>
       <c r="AG84" s="3"/>
       <c r="AH84" s="3"/>
-    </row>
-    <row r="85" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI84" s="3"/>
+    </row>
+    <row r="85" spans="1:35" ht="15.75" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -5891,8 +6009,9 @@
       <c r="AF85" s="3"/>
       <c r="AG85" s="3"/>
       <c r="AH85" s="3"/>
-    </row>
-    <row r="86" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI85" s="3"/>
+    </row>
+    <row r="86" spans="1:35" ht="15.75" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -5927,8 +6046,9 @@
       <c r="AF86" s="3"/>
       <c r="AG86" s="3"/>
       <c r="AH86" s="3"/>
-    </row>
-    <row r="87" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI86" s="3"/>
+    </row>
+    <row r="87" spans="1:35" ht="15.75" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -5963,8 +6083,9 @@
       <c r="AF87" s="3"/>
       <c r="AG87" s="3"/>
       <c r="AH87" s="3"/>
-    </row>
-    <row r="88" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI87" s="3"/>
+    </row>
+    <row r="88" spans="1:35" ht="15.75" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -5999,8 +6120,9 @@
       <c r="AF88" s="3"/>
       <c r="AG88" s="3"/>
       <c r="AH88" s="3"/>
-    </row>
-    <row r="89" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI88" s="3"/>
+    </row>
+    <row r="89" spans="1:35" ht="15.75" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -6035,8 +6157,9 @@
       <c r="AF89" s="3"/>
       <c r="AG89" s="3"/>
       <c r="AH89" s="3"/>
-    </row>
-    <row r="90" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI89" s="3"/>
+    </row>
+    <row r="90" spans="1:35" ht="15.75" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -6071,8 +6194,9 @@
       <c r="AF90" s="3"/>
       <c r="AG90" s="3"/>
       <c r="AH90" s="3"/>
-    </row>
-    <row r="91" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI90" s="3"/>
+    </row>
+    <row r="91" spans="1:35" ht="15.75" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -6107,8 +6231,9 @@
       <c r="AF91" s="3"/>
       <c r="AG91" s="3"/>
       <c r="AH91" s="3"/>
-    </row>
-    <row r="92" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI91" s="3"/>
+    </row>
+    <row r="92" spans="1:35" ht="15.75" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -6143,8 +6268,9 @@
       <c r="AF92" s="3"/>
       <c r="AG92" s="3"/>
       <c r="AH92" s="3"/>
-    </row>
-    <row r="93" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI92" s="3"/>
+    </row>
+    <row r="93" spans="1:35" ht="15.75" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -6179,8 +6305,9 @@
       <c r="AF93" s="3"/>
       <c r="AG93" s="3"/>
       <c r="AH93" s="3"/>
-    </row>
-    <row r="94" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI93" s="3"/>
+    </row>
+    <row r="94" spans="1:35" ht="15.75" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -6215,8 +6342,9 @@
       <c r="AF94" s="3"/>
       <c r="AG94" s="3"/>
       <c r="AH94" s="3"/>
-    </row>
-    <row r="95" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI94" s="3"/>
+    </row>
+    <row r="95" spans="1:35" ht="15.75" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -6251,8 +6379,9 @@
       <c r="AF95" s="3"/>
       <c r="AG95" s="3"/>
       <c r="AH95" s="3"/>
-    </row>
-    <row r="96" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI95" s="3"/>
+    </row>
+    <row r="96" spans="1:35" ht="15.75" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -6287,8 +6416,9 @@
       <c r="AF96" s="3"/>
       <c r="AG96" s="3"/>
       <c r="AH96" s="3"/>
-    </row>
-    <row r="97" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI96" s="3"/>
+    </row>
+    <row r="97" spans="1:35" ht="15.75" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -6323,8 +6453,9 @@
       <c r="AF97" s="3"/>
       <c r="AG97" s="3"/>
       <c r="AH97" s="3"/>
-    </row>
-    <row r="98" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI97" s="3"/>
+    </row>
+    <row r="98" spans="1:35" ht="15.75" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -6359,8 +6490,9 @@
       <c r="AF98" s="3"/>
       <c r="AG98" s="3"/>
       <c r="AH98" s="3"/>
-    </row>
-    <row r="99" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI98" s="3"/>
+    </row>
+    <row r="99" spans="1:35" ht="15.75" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -6395,8 +6527,9 @@
       <c r="AF99" s="3"/>
       <c r="AG99" s="3"/>
       <c r="AH99" s="3"/>
-    </row>
-    <row r="100" spans="1:34" ht="15.75" customHeight="1">
+      <c r="AI99" s="3"/>
+    </row>
+    <row r="100" spans="1:35" ht="15.75" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -6431,6 +6564,7 @@
       <c r="AF100" s="3"/>
       <c r="AG100" s="3"/>
       <c r="AH100" s="3"/>
+      <c r="AI100" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
Add farther typo fallback for mobile, email, nic and other father fields
</commit_message>
<xml_diff>
--- a/StudentMasterDatalocal system.xlsx
+++ b/StudentMasterDatalocal system.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="864" windowWidth="22428" windowHeight="8664" firstSheet="5" activeTab="5"/>
+    <workbookView xWindow="420" yWindow="864" windowWidth="22428" windowHeight="8664" firstSheet="5" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Branch" sheetId="1" r:id="rId1"/>
@@ -257,9 +257,6 @@
     <t>is_living</t>
   </si>
   <si>
-    <t>father</t>
-  </si>
-  <si>
     <t>MARRIED/UNMARRIED</t>
   </si>
   <si>
@@ -501,6 +498,9 @@
   </si>
   <si>
     <t>Bergur</t>
+  </si>
+  <si>
+    <t>farther</t>
   </si>
 </sst>
 </file>
@@ -2541,31 +2541,31 @@
         <v>42</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>28</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>21</v>
@@ -2617,16 +2617,16 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="M2" s="3">
         <v>1</v>
@@ -2638,13 +2638,13 @@
         <v>1</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Q2" s="3">
         <v>1</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="S2" s="3">
         <v>1</v>
@@ -2670,19 +2670,19 @@
       <c r="AB2" s="3"/>
       <c r="AC2" s="3"/>
       <c r="AD2" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="AE2" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="AF2" s="10" t="s">
         <v>148</v>
-      </c>
-      <c r="AE2" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="AF2" s="10" t="s">
-        <v>149</v>
       </c>
       <c r="AG2" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AH2" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AI2" s="3" t="s">
         <v>54</v>
@@ -2698,7 +2698,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
@@ -2709,25 +2709,25 @@
         <v>2</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q3" s="3">
         <v>2</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="S3" s="3">
         <v>2</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="U3" s="3">
         <v>2</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -2738,14 +2738,14 @@
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
       <c r="AE3" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AF3" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AG3" s="3"/>
       <c r="AH3" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AI3" s="3"/>
     </row>
@@ -2780,13 +2780,13 @@
         <v>3</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="U4" s="3">
         <v>3</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -2797,14 +2797,14 @@
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
       <c r="AE4" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AF4" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AI4" s="3"/>
     </row>
@@ -2831,13 +2831,13 @@
         <v>4</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="U5" s="3">
         <v>4</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -2848,7 +2848,7 @@
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
       <c r="AE5" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
@@ -2878,13 +2878,13 @@
         <v>5</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="U6" s="3">
         <v>5</v>
       </c>
       <c r="V6" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
@@ -2923,13 +2923,13 @@
         <v>6</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U7" s="3">
         <v>6</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
@@ -2968,13 +2968,13 @@
         <v>7</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U8" s="3">
         <v>7</v>
       </c>
       <c r="V8" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -3013,13 +3013,13 @@
         <v>8</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="U9" s="3">
         <v>8</v>
       </c>
       <c r="V9" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
@@ -3058,13 +3058,13 @@
         <v>9</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="U10" s="3">
         <v>9</v>
       </c>
       <c r="V10" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
@@ -3103,13 +3103,13 @@
         <v>10</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U11" s="3">
         <v>10</v>
       </c>
       <c r="V11" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
@@ -3150,7 +3150,7 @@
         <v>11</v>
       </c>
       <c r="V12" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
@@ -3191,7 +3191,7 @@
         <v>12</v>
       </c>
       <c r="V13" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
@@ -3232,7 +3232,7 @@
         <v>13</v>
       </c>
       <c r="V14" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
@@ -3273,7 +3273,7 @@
         <v>14</v>
       </c>
       <c r="V15" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
@@ -3314,7 +3314,7 @@
         <v>15</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
@@ -3355,7 +3355,7 @@
         <v>16</v>
       </c>
       <c r="V17" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
@@ -3396,7 +3396,7 @@
         <v>17</v>
       </c>
       <c r="V18" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
@@ -3437,7 +3437,7 @@
         <v>18</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -3478,7 +3478,7 @@
         <v>19</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
@@ -3519,7 +3519,7 @@
         <v>20</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
@@ -3560,7 +3560,7 @@
         <v>21</v>
       </c>
       <c r="V22" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
@@ -3601,7 +3601,7 @@
         <v>22</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
@@ -3642,7 +3642,7 @@
         <v>23</v>
       </c>
       <c r="V24" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="W24" s="3"/>
       <c r="X24" s="3"/>
@@ -3683,7 +3683,7 @@
         <v>24</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="W25" s="3"/>
       <c r="X25" s="3"/>
@@ -3724,7 +3724,7 @@
         <v>25</v>
       </c>
       <c r="V26" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="W26" s="3"/>
       <c r="X26" s="3"/>
@@ -3765,7 +3765,7 @@
         <v>26</v>
       </c>
       <c r="V27" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="W27" s="3"/>
       <c r="X27" s="3"/>
@@ -3806,7 +3806,7 @@
         <v>27</v>
       </c>
       <c r="V28" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W28" s="3"/>
       <c r="X28" s="3"/>
@@ -3847,7 +3847,7 @@
         <v>28</v>
       </c>
       <c r="V29" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="W29" s="3"/>
       <c r="X29" s="3"/>
@@ -3888,7 +3888,7 @@
         <v>29</v>
       </c>
       <c r="V30" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="W30" s="3"/>
       <c r="X30" s="3"/>
@@ -3929,7 +3929,7 @@
         <v>30</v>
       </c>
       <c r="V31" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="W31" s="3"/>
       <c r="X31" s="3"/>
@@ -3970,7 +3970,7 @@
         <v>31</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="W32" s="3"/>
       <c r="X32" s="3"/>
@@ -4011,7 +4011,7 @@
         <v>32</v>
       </c>
       <c r="V33" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="W33" s="3"/>
       <c r="X33" s="3"/>
@@ -4052,7 +4052,7 @@
         <v>33</v>
       </c>
       <c r="V34" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
@@ -4093,7 +4093,7 @@
         <v>34</v>
       </c>
       <c r="V35" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="W35" s="3"/>
       <c r="X35" s="3"/>
@@ -4134,7 +4134,7 @@
         <v>35</v>
       </c>
       <c r="V36" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="W36" s="3"/>
       <c r="X36" s="3"/>
@@ -4175,7 +4175,7 @@
         <v>36</v>
       </c>
       <c r="V37" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="W37" s="3"/>
       <c r="X37" s="3"/>
@@ -4216,7 +4216,7 @@
         <v>37</v>
       </c>
       <c r="V38" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="W38" s="3"/>
       <c r="X38" s="3"/>
@@ -4257,7 +4257,7 @@
         <v>38</v>
       </c>
       <c r="V39" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="W39" s="3"/>
       <c r="X39" s="3"/>
@@ -4298,7 +4298,7 @@
         <v>39</v>
       </c>
       <c r="V40" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W40" s="3"/>
       <c r="X40" s="3"/>
@@ -4339,7 +4339,7 @@
         <v>40</v>
       </c>
       <c r="V41" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="W41" s="3"/>
       <c r="X41" s="3"/>
@@ -4380,7 +4380,7 @@
         <v>41</v>
       </c>
       <c r="V42" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -4421,7 +4421,7 @@
         <v>42</v>
       </c>
       <c r="V43" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="W43" s="3"/>
       <c r="X43" s="3"/>
@@ -4462,7 +4462,7 @@
         <v>43</v>
       </c>
       <c r="V44" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="W44" s="3"/>
       <c r="X44" s="3"/>
@@ -4503,7 +4503,7 @@
         <v>44</v>
       </c>
       <c r="V45" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="W45" s="3"/>
       <c r="X45" s="3"/>
@@ -4544,7 +4544,7 @@
         <v>45</v>
       </c>
       <c r="V46" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W46" s="3"/>
       <c r="X46" s="3"/>
@@ -4585,7 +4585,7 @@
         <v>46</v>
       </c>
       <c r="V47" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="W47" s="3"/>
       <c r="X47" s="3"/>
@@ -4626,7 +4626,7 @@
         <v>47</v>
       </c>
       <c r="V48" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -6711,7 +6711,7 @@
         <v>8524</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
@@ -6722,10 +6722,10 @@
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG2" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="AG2" s="3" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:33" ht="14.4">
@@ -6733,7 +6733,7 @@
         <v>8524</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
@@ -6751,7 +6751,7 @@
         <v>8524</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>

</xml_diff>